<commit_message>
feat(security): SEC-10 — R-SEC20/7/21 amends, R-SEC22 CCVR conflict and scope notes, security_v05
</commit_message>
<xml_diff>
--- a/features/security/sandbox/delivery/FM-WI-FSM-036-A01 STLA 測試用例規範與結果_SWQT STLA Test Case Specification & Result_SWQT_Security_20260917.xlsx
+++ b/features/security/sandbox/delivery/FM-WI-FSM-036-A01 STLA 測試用例規範與結果_SWQT STLA Test Case Specification & Result_SWQT_Security_20260917.xlsx
@@ -8211,7 +8211,8 @@
 sibling axis: verification outcome; rule 1,3 of SEC-04 4.2
 channel_feasible: Y/Y
 asset: X-h — 3. PENDING: X-h log keyword
-apk pairing: fotaMcpuCertTestBrokenCert (apk_pairing.tsv)</t>
+apk pairing: fotaMcpuCertTestBrokenCert (apk_pairing.tsv)
+scope: service-level validation; reprogramming rejection owned by SWDL (CCVR Cert Val CS.98 rationale)</t>
         </is>
       </c>
     </row>
@@ -8504,7 +8505,8 @@
 sibling axis: subject match; rule 1,3 of SEC-04 4.2
 channel_feasible: Y/N
 asset: X-e — 3. PENDING: X-e wrong-subject certificate + trigger
-asset: X-h — 3. PENDING: X-h log keyword</t>
+asset: X-h — 3. PENDING: X-h log keyword
+scope: service-level validation; reprogramming rejection owned by SWDL (CCVR Cert Val CS.98 rationale)</t>
         </is>
       </c>
     </row>
@@ -8797,7 +8799,8 @@
 sibling axis: issuer match; rule 1,3 of SEC-04 4.2
 channel_feasible: Y/Y
 asset: X-e — 3. PENDING: X-e wrong-issuer certificate + trigger
-asset: X-h — 3. PENDING: X-h log keyword</t>
+asset: X-h — 3. PENDING: X-h log keyword
+scope: service-level validation; reprogramming rejection owned by SWDL (CCVR Cert Val CS.98 rationale)</t>
         </is>
       </c>
     </row>
@@ -9086,7 +9089,8 @@
 sibling axis: extension value; rule 1,3 of SEC-04 4.2
 channel_feasible: Y/N
 asset: X-e — 2. PENDING: X-e OID certificate + trigger
-asset: X-h — 2. PENDING: X-h log keyword</t>
+asset: X-h — 2. PENDING: X-h log keyword
+scope: service-level validation; reprogramming rejection owned by SWDL (CCVR Cert Val CS.98 rationale)</t>
         </is>
       </c>
     </row>
@@ -9230,7 +9234,9 @@
 sibling axis: revocation outcome; rule 1,3 of SEC-04 4.2
 channel_feasible: Y/Y
 asset: X-e — 2. PENDING: X-e revoked certificate + trigger
-asset: X-h — 2. PENDING: X-h log keyword</t>
+asset: X-h — 2. PENDING: X-h log keyword
+conflict: 529/383/532/539 — DCL not deployed; unresolved per CCVR Mapping notes row 10
+scope: service-level validation; reprogramming rejection owned by SWDL (CCVR Cert Val CS.98 rationale)</t>
         </is>
       </c>
     </row>
@@ -9369,7 +9375,9 @@
           <t xml:space="preserve">source: 037 SWE1-CertProvider-004 Requirement Description and Verification Criteria
 Polarion: NRL-349387
 sibling axis: verification path; rule 1 of SEC-04 4.2
-channel_feasible: Y/Y</t>
+channel_feasible: Y/Y
+conflict: 529/383/532/539 — DCL not deployed; unresolved per CCVR Mapping notes row 10
+scope: service-level validation; reprogramming rejection owned by SWDL (CCVR Cert Val CS.98 rationale)</t>
         </is>
       </c>
     </row>
@@ -9509,7 +9517,9 @@
 sibling axis: revocation outcome; rule 1,3 of SEC-04 4.2
 channel_feasible: Y/Y
 asset: X-e — 1. PENDING: X-e revoked certificate at the distribution point + trigger
-asset: X-h — 1. PENDING: X-h log keyword</t>
+asset: X-h — 1. PENDING: X-h log keyword
+conflict: 529/383/532/539 — DCL not deployed; unresolved per CCVR Mapping notes row 10
+scope: service-level validation; reprogramming rejection owned by SWDL (CCVR Cert Val CS.98 rationale)</t>
         </is>
       </c>
     </row>
@@ -9647,7 +9657,9 @@
           <t xml:space="preserve">source: 037 SWE1-CertProvider-005 Requirement Description and Verification Criteria
 Polarion: NRL-349388
 sibling axis: storage side effect; rule 1 of SEC-04 4.2
-channel_feasible: Y/Y</t>
+channel_feasible: Y/Y
+conflict: 529/383/532/539 — DCL not deployed; unresolved per CCVR Mapping notes row 10
+scope: service-level validation; reprogramming rejection owned by SWDL (CCVR Cert Val CS.98 rationale)</t>
         </is>
       </c>
     </row>
@@ -10483,7 +10495,8 @@
           <t xml:space="preserve">source: 037 SWE1-CertProvider-007 Requirement Description and Verification Criteria
 Polarion: NRL-349390
 sibling axis: store presence; rule 1 of SEC-04 4.2
-channel_feasible: Y/Y</t>
+channel_feasible: Y/Y
+conflict: 543/546 vs 226; 517 vs 520 — root &amp; CA lifecycle; unresolved per CCVR Mapping notes row 12</t>
         </is>
       </c>
     </row>
@@ -10629,7 +10642,8 @@
 sibling axis: persistence after factory reset; rule 4,5 of SEC-04 4.2
 channel_feasible: Y/Y
 asset: X-e — 3. PENDING: X-e valid leaf certificate + trigger
-asset: X-h — 3. PENDING: X-h log keyword</t>
+asset: X-h — 3. PENDING: X-h log keyword
+conflict: 543/546 vs 226; 517 vs 520 — root &amp; CA lifecycle; unresolved per CCVR Mapping notes row 12</t>
         </is>
       </c>
     </row>
@@ -10770,7 +10784,8 @@
           <t xml:space="preserve">source: 037 SWE1-CertProvider-009 Requirement Description and Verification Criteria
 Polarion: NRL-349392
 sibling axis: configuration version; rule 1,2 of SEC-04 4.2
-channel_feasible: Y/Y</t>
+channel_feasible: Y/Y
+conflict: 543/546 vs 226; 517 vs 520 — root &amp; CA lifecycle; unresolved per CCVR Mapping notes row 12</t>
         </is>
       </c>
     </row>
@@ -10913,7 +10928,8 @@
 sibling axis: configuration version; rule 1,2 of SEC-04 4.2
 channel_feasible: Y/Y
 asset: X-c — 2. PENDING: X-c NR1L production certificate + trigger
-asset: X-h — 2. PENDING: X-h log keyword</t>
+asset: X-h — 2. PENDING: X-h log keyword
+conflict: 543/546 vs 226; 517 vs 520 — root &amp; CA lifecycle; unresolved per CCVR Mapping notes row 12</t>
         </is>
       </c>
     </row>
@@ -10948,7 +10964,7 @@
       <c r="I31" s="81" t="inlineStr">
         <is>
           <t xml:space="preserve">The Cert Provider feature shall provide standardized client interfaces to support both Java and Native clients.
-(Java client invokes the Binder interface for certificate validation (document review))</t>
+(Java client invokes the Binder interface for certificate validation (document review + log observation))</t>
         </is>
       </c>
       <c r="J31" s="81" t="inlineStr">
@@ -11094,7 +11110,7 @@
       <c r="I32" s="81" t="inlineStr">
         <is>
           <t xml:space="preserve">The Cert Provider feature shall provide standardized client interfaces to support both Java and Native clients.
-(Native client uses the libCertProvider C++ API for leaf verification (document review))</t>
+(Native client uses the libCertProvider C++ API for leaf verification (document review + log observation))</t>
         </is>
       </c>
       <c r="J32" s="81" t="inlineStr">
@@ -13693,7 +13709,8 @@
 source: Z1 IntegrationTests/PythonTests/KeysInstallationTests/test_java_integration.py (instrument command verbatim)
 sibling axis: key state; rule 1,3 of SEC-04 4.2
 channel_feasible: Y/Y
-apk pairing: encryptDecryptNormalFlow (apk_pairing.tsv)</t>
+apk pairing: encryptDecryptNormalFlow (apk_pairing.tsv)
+conflict: 376/509/511 vs 510 vs 514 — key strength; unresolved per CCVR Mapping notes row 14</t>
         </is>
       </c>
     </row>
@@ -13833,7 +13850,8 @@
 source: Z1 IntegrationTests/PythonTests/KeysInstallationTests/test_java_integration.py (instrument command verbatim)
 sibling axis: key state; rule 1,3 of SEC-04 4.2
 channel_feasible: Y/Y
-apk pairing: encryptDecryptNormalFlow (apk_pairing.tsv)</t>
+apk pairing: encryptDecryptNormalFlow (apk_pairing.tsv)
+conflict: 376/509/511 vs 510 vs 514 — key strength; unresolved per CCVR Mapping notes row 14</t>
         </is>
       </c>
     </row>
@@ -13969,7 +13987,8 @@
 sibling axis: client authorization; rule 1,3 of SEC-04 4.2
 channel_feasible: Y/Y
 asset: X-f-2 — 1. PENDING: X-f-2 KeyInstall status test runner
-asset: X-f-2 — 1. PENDING: X-f-2 KeyInstall status test runner</t>
+asset: X-f-2 — 1. PENDING: X-f-2 KeyInstall status test runner
+conflict: 376/509/511 vs 510 vs 514 — key strength; unresolved per CCVR Mapping notes row 14</t>
         </is>
       </c>
     </row>
@@ -14109,7 +14128,8 @@
 channel_feasible: Y/Y
 asset: X-f-2 — 1. PENDING: X-f-2 KeyInstall status test runner
 asset: X-f-2 — 1. PENDING: X-f-2 KeyInstall status test runner
-asset: X-h — 2. PENDING: X-h log keyword</t>
+asset: X-h — 2. PENDING: X-h log keyword
+conflict: 376/509/511 vs 510 vs 514 — key strength; unresolved per CCVR Mapping notes row 14</t>
         </is>
       </c>
     </row>
@@ -20456,7 +20476,8 @@
         <is>
           <t xml:space="preserve">source: 037 SYSAD_SEC_ECUCERT_ECUCERT_SRV_EXPORTCSR_INTF Requirement Description and Verification Criteria
 sibling axis: export target; rule 1 of SEC-04 4.2
-channel_feasible: Y/Y</t>
+channel_feasible: Y/Y
+conflict: 562~565 — CSR format evidence pending; unresolved per CCVR Mapping notes row 15</t>
         </is>
       </c>
     </row>
@@ -20870,7 +20891,8 @@
 sibling axis: input range; rule 1 of SEC-04 4.2
 channel_feasible: Y/Y
 asset: X-l — 1. PENDING: X-l SWDL decryption test entry point
-asset: X-l — 1. PENDING: X-l SWDL decryption test entry point</t>
+asset: X-l — 1. PENDING: X-l SWDL decryption test entry point
+conflict: 344 vs Auth-Prog item 7 — rollback; unresolved per CCVR Mapping notes row 13</t>
         </is>
       </c>
     </row>
@@ -21007,7 +21029,8 @@
 sibling axis: decryption outcome; rule 1,3 of SEC-04 4.2
 channel_feasible: Y/Y
 asset: X-l — 1. PENDING: X-l SWDL decryption test entry point
-asset: X-l — 1. PENDING: X-l SWDL decryption test entry point</t>
+asset: X-l — 1. PENDING: X-l SWDL decryption test entry point
+conflict: 344 vs Auth-Prog item 7 — rollback; unresolved per CCVR Mapping notes row 13</t>
         </is>
       </c>
     </row>
@@ -21144,7 +21167,8 @@
 sibling axis: decryption outcome; rule 1,3 of SEC-04 4.2
 channel_feasible: Y/Y
 asset: X-l — 1. PENDING: X-l SWDL decryption test entry point
-asset: X-l — 1. PENDING: X-l SWDL decryption test entry point</t>
+asset: X-l — 1. PENDING: X-l SWDL decryption test entry point
+conflict: 344 vs Auth-Prog item 7 — rollback; unresolved per CCVR Mapping notes row 13</t>
         </is>
       </c>
     </row>
@@ -21281,7 +21305,8 @@
 sibling axis: input range; rule 1 of SEC-04 4.2
 channel_feasible: Y/Y
 asset: X-l — 1. PENDING: X-l SWDL verification test entry point
-asset: X-l — 1. PENDING: X-l SWDL verification test entry point</t>
+asset: X-l — 1. PENDING: X-l SWDL verification test entry point
+conflict: 344 vs Auth-Prog item 7 — rollback; unresolved per CCVR Mapping notes row 13</t>
         </is>
       </c>
     </row>
@@ -21415,9 +21440,10 @@
       <c r="AH105" s="83" t="inlineStr">
         <is>
           <t xml:space="preserve">source: 037 SWE1-SRA-SECURITY-SWDL-004 Requirement Description and Verification Criteria
-source: CCVR Auth-Prog CS.93 evidence rows 3/5/6/7/8; response byte 4 bit field per CS.00102 SYS-RA-CS00102-685
+source: CCVR Auth-Prog CS.93 evidence items 3/5/6/7/8; response byte 4 bit field per CS.00102 SYS-RA-CS00102-685
 sibling axis: verification outcome; rule 1,3 of SEC-04 4.2
-channel_feasible: Y/Y</t>
+channel_feasible: Y/Y
+conflict: 344 vs Auth-Prog item 7 — rollback; unresolved per CCVR Mapping notes row 13</t>
         </is>
       </c>
     </row>
@@ -21551,9 +21577,10 @@
       <c r="AH106" s="83" t="inlineStr">
         <is>
           <t xml:space="preserve">source: 037 SWE1-SRA-SECURITY-SWDL-004 Requirement Description and Verification Criteria
-source: CCVR Auth-Prog CS.93 evidence rows 3/5/6/7/8; response byte 4 bit field per CS.00102 SYS-RA-CS00102-685
+source: CCVR Auth-Prog CS.93 evidence items 3/5/6/7/8; response byte 4 bit field per CS.00102 SYS-RA-CS00102-685
 sibling axis: verification outcome; rule 1,3 of SEC-04 4.2
-channel_feasible: Y/Y</t>
+channel_feasible: Y/Y
+conflict: 344 vs Auth-Prog item 7 — rollback; unresolved per CCVR Mapping notes row 13</t>
         </is>
       </c>
     </row>

</xml_diff>